<commit_message>
Add 30y MOEX tenor, fix interpolation
</commit_message>
<xml_diff>
--- a/data/gcurve_2026-07-31.xlsx
+++ b/data/gcurve_2026-07-31.xlsx
@@ -433,7 +433,7 @@
         <v>0.0028</v>
       </c>
       <c r="B2" t="n">
-        <v>13.827312</v>
+        <v>13.59</v>
       </c>
     </row>
     <row r="3">
@@ -441,7 +441,7 @@
         <v>0.0417</v>
       </c>
       <c r="B3" t="n">
-        <v>13.789968</v>
+        <v>13.59</v>
       </c>
     </row>
     <row r="4">
@@ -449,7 +449,7 @@
         <v>0.1667</v>
       </c>
       <c r="B4" t="n">
-        <v>13.669968</v>
+        <v>13.59</v>
       </c>
     </row>
     <row r="5">
@@ -577,7 +577,7 @@
         <v>25</v>
       </c>
       <c r="B20" t="n">
-        <v>16.06</v>
+        <v>16.025</v>
       </c>
     </row>
   </sheetData>

</xml_diff>